<commit_message>
Close Uttarakhand's last gap: Roads/Potholes via Nagar Nigam Dehradun's PWD
nagarnigamdehradun.com's Public Work Department page names a real
Executive Engineer (Rajit Kothyal) with a direct phone number. The
page has no explicit "handles roads/potholes" sentence, so this
relies on "Public Work Department" being standard, well-established
Indian municipal terminology -- disclosed honestly in the record
itself, same evidentiary tier as other well-established-geography
facts already used in this project.

Uttarakhand now has full 4/4 coverage -- the 3rd state (with
Jharkhand and Chandigarh) fully closed this session.

Rebuilt the knowledge base and real embeddings: 260->261 records,
923->926 chunks in the live ChromaDB index. Updates the vector-store
test's hardcoded chunk-count assertion to match.
</commit_message>
<xml_diff>
--- a/Data_Coverage_Dashboard.xlsx
+++ b/Data_Coverage_Dashboard.xlsx
@@ -538,7 +538,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="9">
@@ -3350,7 +3350,7 @@
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
         <v>0</v>
@@ -6110,7 +6110,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>

</xml_diff>